<commit_message>
notas de credito actualizacion
</commit_message>
<xml_diff>
--- a/data/NC_semanal.xlsx
+++ b/data/NC_semanal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\Desktop\MetrovaloresApp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1521EB4-368B-44C0-90B6-CB9A77B3B502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0949809-FD2E-476D-BBCE-10DA7EEB1B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{9E78C8B1-ED59-4A81-8FF9-F1A88ED1C1A0}"/>
   </bookViews>
@@ -959,311 +959,311 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>26689.62</v>
+        <v>48934.9</v>
       </c>
       <c r="B2" s="2">
-        <v>98.45</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>20016.41</v>
+        <v>235231.13</v>
       </c>
       <c r="B3" s="2">
-        <v>98.45</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>24155.49</v>
+        <v>1482.81</v>
       </c>
       <c r="B4" s="2">
-        <v>98.45</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
-        <v>4816.92</v>
+        <v>108866.76</v>
       </c>
       <c r="B5" s="2">
-        <v>98</v>
+        <v>98.71</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
-        <v>762.49</v>
+        <v>33498.839999999997</v>
       </c>
       <c r="B6" s="2">
-        <v>97</v>
+        <v>98.58</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <v>35270.269999999997</v>
+        <v>494.88</v>
       </c>
       <c r="B7" s="2">
-        <v>98.5</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>20706.03</v>
+        <v>16648.47</v>
       </c>
       <c r="B8" s="2">
-        <v>98.45</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
-        <v>1155398.49</v>
+        <v>1865.45</v>
       </c>
       <c r="B9" s="2">
-        <v>98.844999999999999</v>
+        <v>98.4</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
-        <v>135163.28</v>
+        <v>19795.189999999999</v>
       </c>
       <c r="B10" s="2">
-        <v>98.7</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
-        <v>3138.86</v>
+        <v>7476.27</v>
       </c>
       <c r="B11" s="2">
-        <v>98.3</v>
+        <v>98.555000000000007</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
-        <v>44941.45</v>
+        <v>47956.04</v>
       </c>
       <c r="B12" s="2">
-        <v>98.56</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
-        <v>2166.9499999999998</v>
+        <v>60000</v>
       </c>
       <c r="B13" s="2">
-        <v>98</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
-        <v>5896</v>
+        <v>23469.88</v>
       </c>
       <c r="B14" s="2">
-        <v>98.3</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
-        <v>15115.26</v>
+        <v>362143.77</v>
       </c>
       <c r="B15" s="2">
-        <v>98.4</v>
+        <v>98.84</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
-        <v>6226.89</v>
+        <v>11772.54</v>
       </c>
       <c r="B16" s="2">
-        <v>98.35</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
-        <v>267835.90000000002</v>
+        <v>500.98</v>
       </c>
       <c r="B17" s="2">
-        <v>98.75</v>
+        <v>97.85</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
-        <v>2843</v>
+        <v>10828.37</v>
       </c>
       <c r="B18" s="2">
-        <v>98.15</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
-        <v>6188.45</v>
+        <v>2210.5300000000002</v>
       </c>
       <c r="B19" s="2">
-        <v>98.3</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
-        <v>1036.33</v>
+        <v>372794.99</v>
       </c>
       <c r="B20" s="2">
-        <v>98.05</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
-        <v>38382.75</v>
+        <v>278409.51</v>
       </c>
       <c r="B21" s="2">
-        <v>98.6</v>
+        <v>98.84</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
-        <v>20958.439999999999</v>
+        <v>69071.09</v>
       </c>
       <c r="B22" s="2">
-        <v>98.43</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
-        <v>1564.7</v>
+        <v>115227.15</v>
       </c>
       <c r="B23" s="2">
-        <v>98.25</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
-        <v>124427.23</v>
+        <v>7957.6</v>
       </c>
       <c r="B24" s="2">
-        <v>98.75</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
-        <v>243301.58</v>
+        <v>3466.46</v>
       </c>
       <c r="B25" s="2">
-        <v>98.75</v>
+        <v>98.15</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
-        <v>251499.76</v>
+        <v>1957.32</v>
       </c>
       <c r="B26" s="2">
-        <v>98.75</v>
+        <v>98.4</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
-        <v>31113.48</v>
+        <v>42000</v>
       </c>
       <c r="B27" s="2">
-        <v>98.65</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
-        <v>285522.5</v>
+        <v>459.63</v>
       </c>
       <c r="B28" s="2">
-        <v>98.75</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
-        <v>663052.13</v>
+        <v>3315</v>
       </c>
       <c r="B29" s="2">
-        <v>98.82</v>
+        <v>98.25</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
-        <v>25269.17</v>
+        <v>8338.73</v>
       </c>
       <c r="B30" s="2">
-        <v>98.65</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
-        <v>2119.61</v>
+        <v>17233.55</v>
       </c>
       <c r="B31" s="2">
-        <v>98</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
-        <v>345.26</v>
+        <v>175109.11</v>
       </c>
       <c r="B32" s="2">
-        <v>95</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
-        <v>3803.13</v>
+        <v>166583.26</v>
       </c>
       <c r="B33" s="2">
-        <v>98</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
-        <v>20624.91</v>
+        <v>14702.37</v>
       </c>
       <c r="B34" s="2">
-        <v>98.7</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
-        <v>52558.8</v>
+        <v>1356.99</v>
       </c>
       <c r="B35" s="2">
-        <v>98.65</v>
+        <v>98.35</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
-        <v>21757.42</v>
+        <v>20000</v>
       </c>
       <c r="B36" s="2">
-        <v>98.5</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
-        <v>1074.97</v>
+        <v>384343.12</v>
       </c>
       <c r="B37" s="2">
-        <v>98</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
-        <v>1384.49</v>
+        <v>45835.37</v>
       </c>
       <c r="B38" s="2">
-        <v>98</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
-        <v>2046.68</v>
+        <v>5624.79</v>
       </c>
       <c r="B39" s="2">
-        <v>98</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
-        <v>36106.49</v>
+        <v>6319.81</v>
       </c>
       <c r="B40" s="2">
         <v>98.5</v>
@@ -1271,63 +1271,63 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
-        <v>52643.97</v>
+        <v>396.66</v>
       </c>
       <c r="B41" s="2">
-        <v>98.67</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
-        <v>1181.6400000000001</v>
+        <v>20127.849999999999</v>
       </c>
       <c r="B42" s="2">
-        <v>98</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
-        <v>95891.24</v>
+        <v>36374.230000000003</v>
       </c>
       <c r="B43" s="2">
-        <v>98.65</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
-        <v>1650</v>
+        <v>197175.9</v>
       </c>
       <c r="B44" s="2">
-        <v>98.4</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
-        <v>17414.89</v>
+        <v>47091.29</v>
       </c>
       <c r="B45" s="2">
-        <v>98.5</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
-        <v>1503.98</v>
+        <v>2300</v>
       </c>
       <c r="B46" s="2">
-        <v>98.05</v>
+        <v>98.15</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
-        <v>7204</v>
+        <v>432.82</v>
       </c>
       <c r="B47" s="2">
-        <v>98.3</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
-        <v>16302.3</v>
+        <v>2479.02</v>
       </c>
       <c r="B48" s="2">
         <v>98.5</v>
@@ -1335,71 +1335,71 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
-        <v>1082436.73</v>
+        <v>21128</v>
       </c>
       <c r="B49" s="2">
-        <v>98.827500000000001</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
-        <v>2953.45</v>
+        <v>70776.009999999995</v>
       </c>
       <c r="B50" s="2">
-        <v>98.1</v>
+        <v>98.73</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
-        <v>70301.820000000007</v>
+        <v>30359.62</v>
       </c>
       <c r="B51" s="2">
-        <v>98.65</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
-        <v>511235.21</v>
+        <v>67904.17</v>
       </c>
       <c r="B52" s="2">
-        <v>98.77</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
-        <v>665.69</v>
+        <v>7214.29</v>
       </c>
       <c r="B53" s="2">
-        <v>96</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
-        <v>2059.54</v>
+        <v>11886.23</v>
       </c>
       <c r="B54" s="2">
-        <v>98.1</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
-        <v>231.77</v>
+        <v>1280.74</v>
       </c>
       <c r="B55" s="2">
-        <v>94</v>
+        <v>98.35</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
-        <v>1234.6500000000001</v>
+        <v>24442.16</v>
       </c>
       <c r="B56" s="2">
-        <v>98.25</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
-        <v>21800.9</v>
+        <v>25527.54</v>
       </c>
       <c r="B57" s="2">
         <v>98.65</v>
@@ -1407,199 +1407,199 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
-        <v>2600</v>
+        <v>5753.2</v>
       </c>
       <c r="B58" s="2">
-        <v>98.15</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
-        <v>1938.99</v>
+        <v>175342.03</v>
       </c>
       <c r="B59" s="2">
-        <v>98.15</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
-        <v>25171.46</v>
+        <v>4338.12</v>
       </c>
       <c r="B60" s="2">
-        <v>98.65</v>
+        <v>98.655000000000001</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
-        <v>5019.67</v>
+        <v>2753.29</v>
       </c>
       <c r="B61" s="2">
-        <v>98.45</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
-        <v>2158.42</v>
+        <v>103772.28</v>
       </c>
       <c r="B62" s="2">
-        <v>98.1</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
-        <v>3859837.33</v>
+        <v>2024.92</v>
       </c>
       <c r="B63" s="2">
-        <v>99.037099999999995</v>
+        <v>98.4</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
-        <v>4569.1499999999996</v>
+        <v>7413.22</v>
       </c>
       <c r="B64" s="2">
-        <v>98.15</v>
+        <v>98.4</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
-        <v>24588.6</v>
+        <v>19900.63</v>
       </c>
       <c r="B65" s="2">
-        <v>98.5</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
-        <v>179219.07</v>
+        <v>424.76</v>
       </c>
       <c r="B66" s="2">
-        <v>98.77</v>
+        <v>97.4</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
-        <v>90839.44</v>
+        <v>1000</v>
       </c>
       <c r="B67" s="2">
-        <v>98.7</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
-        <v>200893.45</v>
+        <v>955.91</v>
       </c>
       <c r="B68" s="2">
-        <v>98.8</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
-        <v>288884.49</v>
+        <v>442.7</v>
       </c>
       <c r="B69" s="2">
-        <v>98.75</v>
+        <v>98.05</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
-        <v>1135028.31</v>
+        <v>274898.32</v>
       </c>
       <c r="B70" s="2">
-        <v>98.85</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
-        <v>2813.11</v>
+        <v>200000</v>
       </c>
       <c r="B71" s="2">
-        <v>98.15</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
-        <v>1306.54</v>
+        <v>1092.43</v>
       </c>
       <c r="B72" s="2">
-        <v>98.5</v>
+        <v>98.15</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
-        <v>7785.93</v>
+        <v>599.27</v>
       </c>
       <c r="B73" s="2">
-        <v>98.4</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
-        <v>2285.7800000000002</v>
+        <v>116482.59</v>
       </c>
       <c r="B74" s="2">
-        <v>98.2</v>
+        <v>98.82</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
-        <v>4807.04</v>
+        <v>8380.8799999999992</v>
       </c>
       <c r="B75" s="2">
-        <v>98.4</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
-        <v>43495.96</v>
+        <v>7840</v>
       </c>
       <c r="B76" s="2">
-        <v>98.45</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
-        <v>3202.29</v>
+        <v>1254.4000000000001</v>
       </c>
       <c r="B77" s="2">
-        <v>98.2</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
-        <v>20724.939999999999</v>
+        <v>5376.84</v>
       </c>
       <c r="B78" s="2">
-        <v>98.65</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
-        <v>200704.77</v>
+        <v>70788.44</v>
       </c>
       <c r="B79" s="2">
-        <v>98.7</v>
+        <v>98.77</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
-        <v>17066.36</v>
+        <v>9686.7000000000007</v>
       </c>
       <c r="B80" s="2">
-        <v>98.55</v>
+        <v>98.614999999999995</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
-        <v>13174.87</v>
+        <v>7969.67</v>
       </c>
       <c r="B81" s="2">
-        <v>98.55</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
-        <v>39102.800000000003</v>
+        <v>14522.32</v>
       </c>
       <c r="B82" s="2">
         <v>98.5</v>
@@ -1607,79 +1607,79 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
-        <v>8912.41</v>
+        <v>612.55999999999995</v>
       </c>
       <c r="B83" s="2">
-        <v>98.35</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
-        <v>15986.85</v>
+        <v>472.03</v>
       </c>
       <c r="B84" s="2">
-        <v>98.55</v>
+        <v>95</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
-        <v>94643.45</v>
+        <v>1214.4000000000001</v>
       </c>
       <c r="B85" s="2">
-        <v>98.750100000000003</v>
+        <v>98</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
-        <v>1705645.17</v>
+        <v>3558.47</v>
       </c>
       <c r="B86" s="2">
-        <v>98.87</v>
+        <v>98.25</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
-        <v>2377</v>
+        <v>12561.1</v>
       </c>
       <c r="B87" s="2">
-        <v>98.15</v>
+        <v>98.35</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
-        <v>88028.65</v>
+        <v>28589.45</v>
       </c>
       <c r="B88" s="2">
-        <v>98.81</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
-        <v>7000</v>
+        <v>5421.89</v>
       </c>
       <c r="B89" s="2">
-        <v>98.15</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
-        <v>26503.56</v>
+        <v>911.43</v>
       </c>
       <c r="B90" s="2">
-        <v>98.45</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
-        <v>22451.13</v>
+        <v>309.79000000000002</v>
       </c>
       <c r="B91" s="2">
-        <v>98.4</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
-        <v>5590.92</v>
+        <v>8371.8700000000008</v>
       </c>
       <c r="B92" s="2">
         <v>98.35</v>
@@ -1687,111 +1687,111 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
-        <v>90866.89</v>
+        <v>1901.11</v>
       </c>
       <c r="B93" s="2">
-        <v>98.75</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
-        <v>1945.49</v>
+        <v>560621.76</v>
       </c>
       <c r="B94" s="2">
-        <v>98.5</v>
+        <v>98.93</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
-        <v>83790.02</v>
+        <v>45639.28</v>
       </c>
       <c r="B95" s="2">
-        <v>98.75</v>
+        <v>98.78</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
-        <v>926.48</v>
+        <v>10744.41</v>
       </c>
       <c r="B96" s="2">
-        <v>97.5</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
-        <v>10088.51</v>
+        <v>2155.15</v>
       </c>
       <c r="B97" s="2">
-        <v>98.4</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
-        <v>2888.86</v>
+        <v>341.74</v>
       </c>
       <c r="B98" s="2">
-        <v>98.3</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
-        <v>1664845.78</v>
+        <v>15986.71</v>
       </c>
       <c r="B99" s="2">
-        <v>98.97</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
-        <v>704339.53</v>
+        <v>448428.53</v>
       </c>
       <c r="B100" s="2">
-        <v>98.82</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
-        <v>4601.41</v>
+        <v>12169.01</v>
       </c>
       <c r="B101" s="2">
-        <v>98.2</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
-        <v>9571.2199999999993</v>
+        <v>16507.09</v>
       </c>
       <c r="B102" s="2">
-        <v>98.4</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
-        <v>41222.68</v>
+        <v>5635.98</v>
       </c>
       <c r="B103" s="2">
-        <v>98.55</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
-        <v>28670.86</v>
+        <v>1009.65</v>
       </c>
       <c r="B104" s="2">
-        <v>98.5</v>
+        <v>98</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
-        <v>3848.38</v>
+        <v>7093.15</v>
       </c>
       <c r="B105" s="2">
-        <v>98.45</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
-        <v>363091.73</v>
+        <v>50000</v>
       </c>
       <c r="B106" s="2">
         <v>98.75</v>
@@ -1799,519 +1799,519 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
-        <v>2478.75</v>
+        <v>200000</v>
       </c>
       <c r="B107" s="2">
-        <v>98</v>
+        <v>98.87</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
-        <v>1403.85</v>
+        <v>222131.74</v>
       </c>
       <c r="B108" s="2">
-        <v>98</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
-        <v>44424.84</v>
+        <v>97820</v>
       </c>
       <c r="B109" s="2">
-        <v>98.6</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
-        <v>525.21</v>
+        <v>5135.76</v>
       </c>
       <c r="B110" s="2">
-        <v>98.061000000000007</v>
+        <v>98.628500000000003</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
-        <v>2246.09</v>
+        <v>1782.54</v>
       </c>
       <c r="B111" s="2">
-        <v>98.3</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
-        <v>296801.64</v>
+        <v>6550.98</v>
       </c>
       <c r="B112" s="2">
-        <v>98.8</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
-        <v>590.94000000000005</v>
+        <v>145385.34</v>
       </c>
       <c r="B113" s="2">
-        <v>98</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
-        <v>1038</v>
+        <v>163631.20000000001</v>
       </c>
       <c r="B114" s="2">
-        <v>97.15</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
-        <v>2835.75</v>
+        <v>307117.32</v>
       </c>
       <c r="B115" s="2">
-        <v>98.15</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
-        <v>25974.78</v>
+        <v>56906.46</v>
       </c>
       <c r="B116" s="2">
-        <v>98.5</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
-        <v>63893.47</v>
+        <v>83495.67</v>
       </c>
       <c r="B117" s="2">
-        <v>98.7</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
-        <v>2323.06</v>
+        <v>937.77</v>
       </c>
       <c r="B118" s="2">
-        <v>98.1</v>
+        <v>97</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
-        <v>71812.25</v>
+        <v>1238.54</v>
       </c>
       <c r="B119" s="2">
-        <v>98.68</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
-        <v>925.59</v>
+        <v>370.17</v>
       </c>
       <c r="B120" s="2">
-        <v>98.26</v>
+        <v>97.05</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
-        <v>3520.13</v>
+        <v>1668.14</v>
       </c>
       <c r="B121" s="2">
-        <v>98.3</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
-        <v>1287.21</v>
+        <v>154.18</v>
       </c>
       <c r="B122" s="2">
-        <v>98.3</v>
+        <v>94.05</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
-        <v>2819.6</v>
+        <v>41504.33</v>
       </c>
       <c r="B123" s="2">
-        <v>98.3</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
-        <v>1415.58</v>
+        <v>2244.23</v>
       </c>
       <c r="B124" s="2">
-        <v>98.2</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
-        <v>2045.35</v>
+        <v>1253.05</v>
       </c>
       <c r="B125" s="2">
-        <v>98.3</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
-        <v>137195.79999999999</v>
+        <v>139.01</v>
       </c>
       <c r="B126" s="2">
-        <v>98.75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
-        <v>404727.63</v>
+        <v>130245.68</v>
       </c>
       <c r="B127" s="2">
-        <v>98.8</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
-        <v>2000</v>
+        <v>59766.53</v>
       </c>
       <c r="B128" s="2">
-        <v>98.3</v>
+        <v>98.78</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
-        <v>925.96</v>
+        <v>21867.53</v>
       </c>
       <c r="B129" s="2">
-        <v>97.5</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
-        <v>1270.51</v>
+        <v>3028.55</v>
       </c>
       <c r="B130" s="2">
-        <v>98</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
-        <v>2103.46</v>
+        <v>483.95</v>
       </c>
       <c r="B131" s="2">
-        <v>98</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
-        <v>2306.11</v>
+        <v>3557.83</v>
       </c>
       <c r="B132" s="2">
-        <v>98</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
-        <v>2258.6799999999998</v>
+        <v>39675.71</v>
       </c>
       <c r="B133" s="2">
-        <v>98.3</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
-        <v>7812.75</v>
+        <v>107176.93</v>
       </c>
       <c r="B134" s="2">
-        <v>98.3</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
-        <v>5448.32</v>
+        <v>556790.26</v>
       </c>
       <c r="B135" s="2">
-        <v>98.3</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
-        <v>1907.55</v>
+        <v>2407822.91</v>
       </c>
       <c r="B136" s="2">
-        <v>98.1</v>
+        <v>99.04</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
-        <v>20571.79</v>
+        <v>23580.95</v>
       </c>
       <c r="B137" s="2">
-        <v>98.5</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
-        <v>1640.19</v>
+        <v>49002.52</v>
       </c>
       <c r="B138" s="2">
-        <v>98.1</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
-        <v>45196.84</v>
+        <v>200000</v>
       </c>
       <c r="B139" s="2">
-        <v>98.55</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
-        <v>186497.62</v>
+        <v>45429.4</v>
       </c>
       <c r="B140" s="2">
-        <v>98.75</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
-        <v>1619.23</v>
+        <v>65650.92</v>
       </c>
       <c r="B141" s="2">
-        <v>98.1</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
-        <v>43011.14</v>
+        <v>36300</v>
       </c>
       <c r="B142" s="2">
-        <v>98.6</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
-        <v>4253.2299999999996</v>
+        <v>284647.07</v>
       </c>
       <c r="B143" s="2">
-        <v>98.25</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
-        <v>4231.8599999999997</v>
+        <v>275698.44</v>
       </c>
       <c r="B144" s="2">
-        <v>98.35</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
-        <v>61064.23</v>
+        <v>200000</v>
       </c>
       <c r="B145" s="2">
-        <v>98.65</v>
+        <v>99.05</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
-        <v>1500</v>
+        <v>14000</v>
       </c>
       <c r="B146" s="2">
-        <v>98.35</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
-        <v>10746.62</v>
+        <v>1064.92</v>
       </c>
       <c r="B147" s="2">
-        <v>98.55</v>
+        <v>98.655000000000001</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
-        <v>152840.21</v>
+        <v>95000</v>
       </c>
       <c r="B148" s="2">
-        <v>98.75</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
-        <v>8397.85</v>
+        <v>2926.89</v>
       </c>
       <c r="B149" s="2">
-        <v>98.45</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
-        <v>31500</v>
+        <v>11279.64</v>
       </c>
       <c r="B150" s="2">
-        <v>98.55</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
-        <v>563.65</v>
+        <v>14740.77</v>
       </c>
       <c r="B151" s="2">
-        <v>97.5</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
-        <v>770000</v>
+        <v>755.13</v>
       </c>
       <c r="B152" s="2">
-        <v>98.85</v>
+        <v>98.15</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
-        <v>112163.36</v>
+        <v>232976.11</v>
       </c>
       <c r="B153" s="2">
-        <v>98.87</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
-        <v>71571.789999999994</v>
+        <v>12738.86</v>
       </c>
       <c r="B154" s="2">
-        <v>98.7</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
-        <v>450000</v>
+        <v>106032.87</v>
       </c>
       <c r="B155" s="2">
-        <v>98.85</v>
+        <v>98.86</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
-        <v>7814025.6799999997</v>
+        <v>51152.34</v>
       </c>
       <c r="B156" s="2">
-        <v>99.077500000000001</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
-        <v>309219.08</v>
+        <v>9028.93</v>
       </c>
       <c r="B157" s="2">
-        <v>98.8</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
-        <v>14800.07</v>
+        <v>9914.76</v>
       </c>
       <c r="B158" s="2">
-        <v>98.6</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
-        <v>28706.45</v>
+        <v>15118.76</v>
       </c>
       <c r="B159" s="2">
-        <v>98.6</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
-        <v>16355.37</v>
+        <v>33113.15</v>
       </c>
       <c r="B160" s="2">
-        <v>99.6</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
-        <v>16355.37</v>
+        <v>39930.1</v>
       </c>
       <c r="B161" s="2">
-        <v>98.6</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
-        <v>5413.77</v>
+        <v>208732.41</v>
       </c>
       <c r="B162" s="2">
-        <v>98.4</v>
+        <v>98.92</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
-        <v>12625.17</v>
+        <v>2254.75</v>
       </c>
       <c r="B163" s="2">
-        <v>98.6</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
-        <v>2346.65</v>
+        <v>1500</v>
       </c>
       <c r="B164" s="2">
-        <v>98.3</v>
+        <v>98.15</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
-        <v>47223.09</v>
+        <v>530744.86</v>
       </c>
       <c r="B165" s="2">
-        <v>98.7</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
-        <v>20718.060000000001</v>
+        <v>98987.7</v>
       </c>
       <c r="B166" s="2">
-        <v>98.7</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
-        <v>5079.47</v>
+        <v>36551.57</v>
       </c>
       <c r="B167" s="2">
-        <v>98.4</v>
+        <v>98.77</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
-        <v>18211.95</v>
+        <v>3009.25</v>
       </c>
       <c r="B168" s="2">
-        <v>98.4</v>
+        <v>98.67</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
-        <v>1832.53</v>
+        <v>40300.22</v>
       </c>
       <c r="B169" s="2">
-        <v>98.3</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
-        <v>353858.67</v>
+        <v>21892.38</v>
       </c>
       <c r="B170" s="2">
-        <v>98.8</v>
+        <v>98.79</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
-        <v>3429.58</v>
+        <v>1667.11</v>
       </c>
       <c r="B171" s="2">
         <v>98.2</v>
@@ -2319,79 +2319,79 @@
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
-        <v>24269.54</v>
+        <v>27638.720000000001</v>
       </c>
       <c r="B172" s="2">
-        <v>98.55</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
-        <v>37128.67</v>
+        <v>11541.92</v>
       </c>
       <c r="B173" s="2">
-        <v>98.5</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
-        <v>14854.7</v>
+        <v>13183.75</v>
       </c>
       <c r="B174" s="2">
-        <v>98.55</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
-        <v>26745.67</v>
+        <v>4152.09</v>
       </c>
       <c r="B175" s="2">
-        <v>98.5</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
-        <v>22174.91</v>
+        <v>1836.35</v>
       </c>
       <c r="B176" s="2">
-        <v>98.5</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
-        <v>14750.87</v>
+        <v>16169.54</v>
       </c>
       <c r="B177" s="2">
-        <v>98.6</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
-        <v>4232.8599999999997</v>
+        <v>271807.40000000002</v>
       </c>
       <c r="B178" s="2">
-        <v>98.3</v>
+        <v>98.92</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
-        <v>1108.45</v>
+        <v>387717.86</v>
       </c>
       <c r="B179" s="2">
-        <v>98.3</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
-        <v>15000</v>
+        <v>53422.03</v>
       </c>
       <c r="B180" s="2">
-        <v>98.5</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
-        <v>4377.83</v>
+        <v>1972.18</v>
       </c>
       <c r="B181" s="2">
         <v>98</v>
@@ -2399,223 +2399,223 @@
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
-        <v>3586.66</v>
+        <v>23075.97</v>
       </c>
       <c r="B182" s="2">
-        <v>98.3</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
-        <v>24084.15</v>
+        <v>1260.08</v>
       </c>
       <c r="B183" s="2">
-        <v>98.6</v>
+        <v>98.15</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
-        <v>5142.71</v>
+        <v>6212.4</v>
       </c>
       <c r="B184" s="2">
-        <v>98.35</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
-        <v>1663.79</v>
+        <v>10844.35</v>
       </c>
       <c r="B185" s="2">
-        <v>98.3</v>
+        <v>98.815700000000007</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
-        <v>23256.92</v>
+        <v>1726.26</v>
       </c>
       <c r="B186" s="2">
-        <v>98.67</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
-        <v>80000</v>
+        <v>5083.93</v>
       </c>
       <c r="B187" s="2">
-        <v>98.75</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
-        <v>69698.509999999995</v>
+        <v>276115.53999999998</v>
       </c>
       <c r="B188" s="2">
-        <v>98.8</v>
+        <v>99.1</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
-        <v>15758.51</v>
+        <v>106122.21</v>
       </c>
       <c r="B189" s="2">
-        <v>98.5</v>
+        <v>98.87</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
-        <v>163950.1</v>
+        <v>5579.91</v>
       </c>
       <c r="B190" s="2">
-        <v>98.8</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
-        <v>25500.51</v>
+        <v>26374.06</v>
       </c>
       <c r="B191" s="2">
-        <v>98.5</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
-        <v>14612.18</v>
+        <v>159857.13</v>
       </c>
       <c r="B192" s="2">
-        <v>98.6</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" s="2">
-        <v>61311.1</v>
+        <v>7536.98</v>
       </c>
       <c r="B193" s="2">
-        <v>98.8</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
-        <v>16522.150000000001</v>
+        <v>698.9</v>
       </c>
       <c r="B194" s="2">
-        <v>98.5</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
-        <v>40338.76</v>
+        <v>625.94000000000005</v>
       </c>
       <c r="B195" s="2">
-        <v>98.73</v>
+        <v>96.6</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
-        <v>37022.86</v>
+        <v>117966.43</v>
       </c>
       <c r="B196" s="2">
-        <v>98.7</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
-        <v>1419.63</v>
+        <v>810.42</v>
       </c>
       <c r="B197" s="2">
-        <v>98.25</v>
+        <v>98</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
-        <v>9023.66</v>
+        <v>420050.4</v>
       </c>
       <c r="B198" s="2">
-        <v>98.5</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" s="2">
-        <v>10245.16</v>
+        <v>733.27</v>
       </c>
       <c r="B199" s="2">
-        <v>98.55</v>
+        <v>98.25</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" s="2">
-        <v>70929.53</v>
+        <v>1361.11</v>
       </c>
       <c r="B200" s="2">
-        <v>98.8</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201" s="2">
-        <v>298334.96999999997</v>
+        <v>5084.43</v>
       </c>
       <c r="B201" s="2">
-        <v>98.82</v>
+        <v>98.55</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A202" s="2">
-        <v>59764.85</v>
+        <v>106783.62</v>
       </c>
       <c r="B202" s="2">
-        <v>98.75</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="2">
-        <v>4213.6899999999996</v>
+        <v>13443.59</v>
       </c>
       <c r="B203" s="2">
-        <v>98.2</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204" s="2">
-        <v>205343.35999999999</v>
+        <v>19405.29</v>
       </c>
       <c r="B204" s="2">
-        <v>98.9</v>
+        <v>98.910899999999998</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A205" s="2">
-        <v>1305.8599999999999</v>
+        <v>422.76</v>
       </c>
       <c r="B205" s="2">
-        <v>98.25</v>
+        <v>96</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206" s="2">
-        <v>427.85</v>
+        <v>107980.68</v>
       </c>
       <c r="B206" s="2">
-        <v>97.5</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A207" s="2">
-        <v>1637.21</v>
+        <v>188476.74</v>
       </c>
       <c r="B207" s="2">
-        <v>98</v>
+        <v>98.96</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208" s="2">
-        <v>14335.62</v>
+        <v>215960.89</v>
       </c>
       <c r="B208" s="2">
-        <v>98.6</v>
+        <v>98.96</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209" s="2">
-        <v>12257.06</v>
+        <v>9266.89</v>
       </c>
       <c r="B209" s="2">
         <v>98.6</v>
@@ -2623,467 +2623,364 @@
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210" s="2">
-        <v>287464.84999999998</v>
+        <v>2309.12</v>
       </c>
       <c r="B210" s="2">
-        <v>98.8</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A211" s="2">
-        <v>709.37</v>
+        <v>11893.14</v>
       </c>
       <c r="B211" s="2">
-        <v>97</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212" s="2">
-        <v>21914</v>
+        <v>44873.87</v>
       </c>
       <c r="B212" s="2">
-        <v>98.6</v>
+        <v>98.75</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213" s="2">
-        <v>7524.79</v>
+        <v>2012.16</v>
       </c>
       <c r="B213" s="2">
-        <v>98.2</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214" s="2">
-        <v>18801.96</v>
+        <v>1607482.98</v>
       </c>
       <c r="B214" s="2">
-        <v>98.6</v>
+        <v>99.02</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215" s="2">
-        <v>127016.36</v>
+        <v>681.26</v>
       </c>
       <c r="B215" s="2">
-        <v>98.9</v>
+        <v>96</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A216" s="2">
-        <v>2553.02</v>
+        <v>10135.35</v>
       </c>
       <c r="B216" s="2">
-        <v>98</v>
+        <v>98.65</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A217" s="2">
-        <v>1389.9</v>
+        <v>12193.32</v>
       </c>
       <c r="B217" s="2">
-        <v>98</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218" s="2">
-        <v>1236.31</v>
+        <v>9489.57</v>
       </c>
       <c r="B218" s="2">
-        <v>98</v>
+        <v>98.6</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A219" s="2">
-        <v>38797.410000000003</v>
+        <v>28359.09</v>
       </c>
       <c r="B219" s="2">
-        <v>98.55</v>
+        <v>99</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A220" s="2">
-        <v>1864.75</v>
+        <v>32694.87</v>
       </c>
       <c r="B220" s="2">
-        <v>98.4</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A221" s="2">
-        <v>2064.9499999999998</v>
+        <v>38110.1</v>
       </c>
       <c r="B221" s="2">
-        <v>98.3</v>
+        <v>99</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A222" s="2">
-        <v>258317.09</v>
+        <v>409.75</v>
       </c>
       <c r="B222" s="2">
-        <v>98.75</v>
+        <v>95</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A223" s="2">
-        <v>1635.31</v>
+        <v>705.65</v>
       </c>
       <c r="B223" s="2">
-        <v>98.4</v>
+        <v>98</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224" s="2">
-        <v>18948.990000000002</v>
+        <v>38018.42</v>
       </c>
       <c r="B224" s="2">
-        <v>98.4</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225" s="2">
-        <v>5500</v>
+        <v>18700</v>
       </c>
       <c r="B225" s="2">
-        <v>98.5</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226" s="2">
-        <v>51685.31</v>
+        <v>13053.97</v>
       </c>
       <c r="B226" s="2">
-        <v>98.65</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227" s="2">
-        <v>5112.18</v>
+        <v>86766.11</v>
       </c>
       <c r="B227" s="2">
-        <v>98.6</v>
+        <v>99</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" s="2">
-        <v>725.41</v>
+        <v>50000</v>
       </c>
       <c r="B228" s="2">
-        <v>97.6</v>
+        <v>98.92</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229" s="2">
-        <v>8457.14</v>
+        <v>63445</v>
       </c>
       <c r="B229" s="2">
-        <v>98.62</v>
+        <v>98.92</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230" s="2">
-        <v>6393.55</v>
+        <v>30791.040000000001</v>
       </c>
       <c r="B230" s="2">
-        <v>98.5</v>
+        <v>98.82</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231" s="2">
-        <v>101413.65</v>
+        <v>11320.45</v>
       </c>
       <c r="B231" s="2">
-        <v>98.7</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232" s="2">
-        <v>47119.44</v>
+        <v>1335.42</v>
       </c>
       <c r="B232" s="2">
-        <v>98.6</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" s="2">
-        <v>2410.44</v>
+        <v>2882.44</v>
       </c>
       <c r="B233" s="2">
-        <v>98.3</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234" s="2">
-        <v>125.22</v>
+        <v>30363.71</v>
       </c>
       <c r="B234" s="2">
-        <v>93</v>
+        <v>98.83</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235" s="2">
-        <v>2347.98</v>
+        <v>111709.91</v>
       </c>
       <c r="B235" s="2">
-        <v>98.4</v>
+        <v>98.85</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236" s="2">
-        <v>433.85</v>
+        <v>1273.5899999999999</v>
       </c>
       <c r="B236" s="2">
-        <v>97.5</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237" s="2">
-        <v>869.13</v>
+        <v>252256.18</v>
       </c>
       <c r="B237" s="2">
-        <v>97.5</v>
+        <v>99</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238" s="2">
-        <v>51682.44</v>
+        <v>40000</v>
       </c>
       <c r="B238" s="2">
-        <v>98.6</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239" s="2">
-        <v>3000</v>
+        <v>3059.74</v>
       </c>
       <c r="B239" s="2">
-        <v>98.45</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240" s="2">
-        <v>663.12</v>
+        <v>140000</v>
       </c>
       <c r="B240" s="2">
-        <v>98.2</v>
+        <v>98.95</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" s="2">
-        <v>2798.58</v>
+        <v>16215.44</v>
       </c>
       <c r="B241" s="2">
-        <v>98.4</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" s="2">
-        <v>2558339.85</v>
+        <v>2466500.83</v>
       </c>
       <c r="B242" s="2">
-        <v>99.02</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" s="2">
-        <v>360.14</v>
+        <v>170000</v>
       </c>
       <c r="B243" s="2">
-        <v>97.05</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A244" s="2">
-        <v>15728.85</v>
-      </c>
-      <c r="B244" s="2">
-        <v>98.7</v>
-      </c>
+      <c r="A244" s="2"/>
+      <c r="B244" s="2"/>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A245" s="2">
-        <v>1358.01</v>
-      </c>
-      <c r="B245" s="2">
-        <v>98</v>
-      </c>
+      <c r="A245" s="2"/>
+      <c r="B245" s="2"/>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A246" s="2">
-        <v>126588.06</v>
-      </c>
-      <c r="B246" s="2">
-        <v>98.8</v>
-      </c>
+      <c r="A246" s="2"/>
+      <c r="B246" s="2"/>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A247" s="2">
-        <v>169450.53</v>
-      </c>
-      <c r="B247" s="2">
-        <v>98.8</v>
-      </c>
+      <c r="A247" s="2"/>
+      <c r="B247" s="2"/>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A248" s="2">
-        <v>163.05000000000001</v>
-      </c>
-      <c r="B248" s="2">
-        <v>97</v>
-      </c>
+      <c r="A248" s="2"/>
+      <c r="B248" s="2"/>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A249" s="2">
-        <v>15148.57</v>
-      </c>
-      <c r="B249" s="2">
-        <v>98.6</v>
-      </c>
+      <c r="A249" s="2"/>
+      <c r="B249" s="2"/>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A250" s="2">
-        <v>39938.300000000003</v>
-      </c>
-      <c r="B250" s="2">
-        <v>98.8</v>
-      </c>
+      <c r="A250" s="2"/>
+      <c r="B250" s="2"/>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A251" s="2">
-        <v>26802.15</v>
-      </c>
-      <c r="B251" s="2">
-        <v>98.6</v>
-      </c>
+      <c r="A251" s="2"/>
+      <c r="B251" s="2"/>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A252" s="2">
-        <v>603.38</v>
-      </c>
-      <c r="B252" s="2">
-        <v>97.75</v>
-      </c>
+      <c r="A252" s="2"/>
+      <c r="B252" s="2"/>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A253" s="2">
-        <v>23493.85</v>
-      </c>
-      <c r="B253" s="2">
-        <v>98.6</v>
-      </c>
+      <c r="A253" s="2"/>
+      <c r="B253" s="2"/>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A254" s="2">
-        <v>143496.5</v>
-      </c>
-      <c r="B254" s="2">
-        <v>98.8</v>
-      </c>
+      <c r="A254" s="2"/>
+      <c r="B254" s="2"/>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A255" s="2">
-        <v>381526.73</v>
-      </c>
-      <c r="B255" s="2">
-        <v>98.8</v>
-      </c>
+      <c r="A255" s="2"/>
+      <c r="B255" s="2"/>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A256" s="2">
-        <v>957881</v>
-      </c>
-      <c r="B256" s="2">
-        <v>98.93</v>
-      </c>
+      <c r="A256" s="2"/>
+      <c r="B256" s="2"/>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A257" s="2">
-        <v>501534.03</v>
-      </c>
-      <c r="B257" s="2">
-        <v>98.83</v>
-      </c>
+      <c r="A257" s="2"/>
+      <c r="B257" s="2"/>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A258" s="2">
-        <v>142870.43</v>
-      </c>
-      <c r="B258" s="2">
-        <v>98.82</v>
-      </c>
+      <c r="A258" s="2"/>
+      <c r="B258" s="2"/>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A259" s="2">
-        <v>167699.91</v>
-      </c>
-      <c r="B259" s="2">
-        <v>98.8</v>
-      </c>
+      <c r="A259" s="2"/>
+      <c r="B259" s="2"/>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A260" s="2">
-        <v>34954.300000000003</v>
-      </c>
-      <c r="B260" s="3">
-        <v>98.65</v>
-      </c>
+      <c r="A260" s="2"/>
+      <c r="B260" s="3"/>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A261" s="2">
-        <v>4567.87</v>
-      </c>
-      <c r="B261" s="1">
-        <v>98.55</v>
-      </c>
+      <c r="A261" s="2"/>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A262" s="2">
-        <v>14950.12</v>
-      </c>
-      <c r="B262" s="1">
-        <v>98.6</v>
-      </c>
+      <c r="A262" s="2"/>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A263" s="2">
-        <v>252852.9</v>
-      </c>
-      <c r="B263" s="1">
-        <v>98.75</v>
-      </c>
+      <c r="A263" s="2"/>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A264" s="2">
-        <v>10000</v>
-      </c>
-      <c r="B264" s="1">
-        <v>98.45</v>
-      </c>
+      <c r="A264" s="2"/>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A265" s="2">
-        <v>507</v>
-      </c>
-      <c r="B265" s="1">
-        <v>97.5</v>
-      </c>
+      <c r="A265" s="2"/>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A266" s="2">
-        <v>1239.55</v>
-      </c>
-      <c r="B266" s="1">
-        <v>98.1</v>
-      </c>
+      <c r="A266" s="2"/>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A267" s="2">
-        <v>1903.61</v>
-      </c>
-      <c r="B267" s="1">
-        <v>98.3</v>
-      </c>
+      <c r="A267" s="2"/>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" s="2"/>

</xml_diff>